<commit_message>
Update daily sales report 2026-10-04.xlsx to October MTD data
Replace the earlier September-close version of this file (same filename due
to the same preparation date) with the genuinely new October 2026 data: NetSuite
report now covers 01-31 October (MTD, 2 active categories), PPLAY1 pivot shows
2026/Oct (6 active categories), and Amazon figures reflect "Month to date, 1-3
October 2026". B1 updated to "דוח מכירות אוקטובר 2026" since source files now
accumulate from the new month. Total sales (C41): 91,909.56 ILS.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-10-04.xlsx
+++ b/kirill/outputs/2026-10-04.xlsx
@@ -25,9 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="102">
-  <si>
-    <t xml:space="preserve">דוח מכירות ספטמבר 2026</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="102">
+  <si>
+    <t xml:space="preserve">דוח מכירות אוקטובר 2026</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -297,16 +297,16 @@
     <t xml:space="preserve">105 - Pedicure Salons</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: PPlay1.xls, "PPlay1 of uriel (Reporter)", נוצר 04/10/2026 08:43:06, תקופה 2026/Sep (סגירת חודש ספטמבר ממשיכה להתעדכן — קובץ נמסר ב-04/10/2026, היום הרביעי של אוקטובר, אך תוכנו עדיין 2026/Sep. לפי המוסכמה: B1 בגיליון סהכ נשאר "ספטמבר 2026" כל עוד קבצי המקור מציגים את חודש ספטמבר ולא התחילו להצטבר מאוקטובר). שוב בפורמט MHTML ("Excel Web Page", MIME multipart) ולא XLSX/ZIP רגיל — זוהה ע"י `file` שמחזיר "MIME entity, ASCII text". פוענח ע"י email.message_from_binary_file + BeautifulSoup על part[2] (Content-Location "sheet001.htm"), decode windows-1255 — פרסור נקי בניסיון ראשון, אינדקס part[2] אומת מחדש ותואם לימים קודמים. נשלפו 10 שורות קטגוריה שיש להן נתונים עד כה החודש, מתוך 13 הקטגוריות במקרא גיליון Pplay1. 3 קטגוריות נותרות ללא נתונים עדיין החודש (גוד פארם מרכז, 0צרכנים פרטיים, 0שונות; תקין לסגירת חודש, לא נתון חסר — זהה לדוחות הקודמים). לעומת 01/10/2026 (הדוח היומי הקודם): 0בתי מרקחת ₪181,860.0→₪186,065.8, 0פארמים ₪533,408.1→₪639,577.2, סופרפארם ₪454,708.2→₪557,932.5, שופרסל BE ₪71,611.0→₪74,555.9, 0קופות חולים ₪60,089.3→₪60,936.5, אילת BE ₪6,632.0→₪6,632.0 (ללא שינוי) — עלייה נוספת, תקין וצפוי (חשבוניות נוספות שנקלטו למפרעה על חודש שעדיין בתהליך סגירה מלאה). 0מפיצי משנה, הפרכל הפרפארם, זיכויים BE, גוד פארם נותרו ללא שינוי בדיוק (אין תנועה חדשה שנקלטה במקור בפער זה — נבדק ואומת ישירות מול הטקסט הגולמי בקובץ המקור, לא שגיאת פענוח). שורת "Customers" בדוח המקור (₪887,157.2) היא שורת סה"כ-אב ואינה שווה לסכום שורות הקטגוריה (₪1,526,734.6) — תקין וצפוי, כרגיל — לא יובאה. מכר נטו = עמודה B × 0.91 (מקדם קבוע, מאושר ב-kirill.md; חל גם על ערך שלילי).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/Sep (סכום גולמי, MTD)</t>
+    <t xml:space="preserve">Source: PPlay1.xls, "PPlay1 of uriel (Reporter)", נוצר 04/10/2026 09:38:30, תקופה 2026/Oct (חודש אוקטובר 2026 - החודש החדש: קבצי המקור עברו להציג MTD שמצטבר מאוקטובר, ולכן B1 בגיליון סהכ עבר ל"אוקטובר 2026", לפי המוסכמה הקבועה. זהו הדוח היומי הראשון של החודש - צפויה הצטברות MTD נמוכה מאוד (רק 1-4 ימים לתוך החודש) בהשוואה לדוח הקודם שהיה סגירת חודש ספטמבר מלא - זו ירידה צפויה ותקינה, לא נתון חסר ולא שגיאת חישוב). שוב בפורמט MHTML ("Excel Web Page", MIME multipart) ולא XLSX/ZIP רגיל - זוהה ע"י `file` שמחזיר "MIME entity, ASCII text". פוענח ע"י email.message_from_binary_file + BeautifulSoup על part[2] (Content-Location "sheet001.htm"), decode windows-1255 - פרסור נקי בניסיון ראשון, אינדקס part[2] אומת מחדש ותואם לימים קודמים. נשלפו 6 שורות קטגוריה שיש להן נתונים עד כה החודש (0בתי מרקחת, 0פארמים, גוד פארם מרכז, סופרפארם, שופרסל BE, 0קופות חולים), מתוך 13 הקטגוריות במקרא גיליון Pplay1. 7 קטגוריות נותרות ללא נתונים עדיין החודש (0מפיצי משנה, אילת BE, הפרכל הפרפארם, זיכויים BE, גוד פארם, 0צרכנים פרטיים, 0שונות) - תקין לתחילת חודש, לא נתון חסר. גוד פארם מרכז מציגה סכום שלילי (₪-284.7) - זיכוי/החזר שנקלט בתחילת החודש, נבדק ואומת ישירות מול הטקסט הגולמי בקובץ המקור, לא שגיאת פענוח. אין שורת "Customers" (סה"כ-אב) בפלט הגולמי הפעם - השורה היחידה שמכילה את המחרוזת "Customers" היא שורת מטא-דאטה של רשימת שדות ה-pivot ("2026/Oct,Months,Companies,Customers,..."), לא שורת סכום, ולכן אין מה להחריג. מכר נטו = עמודה B × 0.91 (מקדם קבוע, מאושר ב-kirill.md; חל גם על ערך שלילי).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026/Oct (סכום גולמי, MTD)</t>
   </si>
   <si>
     <t xml:space="preserve">הערה</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: CustomSalesbyCustomerSummary929.xlsx, Meditex Group IL, Custom Sales by Customer Summary, 01 September 2026 - 30 September 2026 (סגירת חודש ספטמבר ממשיכה להתעדכן), נמסר 04/10/2026 עבור דוח 04/10/2026. קובץ xlsx תקני (2007+) — נטען ישירות ע"י openpyxl ללא צורך בתיקון קידוד. נשלפו 14 שורות הסיכום (קטגוריה) שיש להן מכירות בחודש, מתוך 28 הקטגוריות במקרא "ריכוז" (14 הקטגוריות הנותרות אין להן מכירות עדיין החודש — תקין, לא נתון חסר — אותן 14 חסרות כמו ב-01/10). לעומת 01/10/2026 (הדוח היומי הקודם): 101 - Factory customers ₪8,755.86→₪8,627.76 (ירידה של ₪128.10, נבדק ואומת ישירות מול הדוח הגולמי — ככל הנראה זיכוי/תיקון חשבונית שנקלט בין הדוחות, לא שגיאת פענוח); שאר 13 הקטגוריות (102, 103, 109, 111, 107, 112, 114, 115, 205, 209, 204, 106, 201) נותרו ללא שינוי בדיוק (אין חשבונית חדשה/מתוקנת לאותו לקוח בפער זה). לא יובאו שורות פירוט חשבוניות/לקוחות-בת מהדוח הגולמי, לפי מוסכמת עבודה. סה"כ שורת "Total" בדוח הגולמי המלא: ₪1,054,442.83 — תואם בדיוק לסכום 14 שורות הקטגוריה שנשלפו (₪1,054,442.83, אומת ידנית, הפרש &lt;0.01₪).</t>
+    <t xml:space="preserve">Source: CustomSalesbyCustomerSummary836.xlsx, Meditex Group IL, Custom Sales by Customer Summary, 01 October 2026 - 31 October 2026 (MTD, החודש החדש - אוקטובר), נמסר 04/10/2026 עבור דוח 04/10/2026. קובץ xlsx תקני (2007+) - נטען ישירות ע"י openpyxl ללא צורך בתיקון קידוד. נשלפו 2 שורות הסיכום (קטגוריה) שיש להן מכירות בחודש עד כה (112 - Kupat Holim Clalit, 114 - IL online), מתוך 28 הקטגוריות במקרא "ריכוז" - 26 הקטגוריות הנותרות אין להן מכירות עדיין החודש, תקין וצפוי לתחילת חודש (רק 1-4 ימים לתוך אוקטובר), לא נתון חסר. לא יובאו שורות פירוט חשבוניות/לקוחות-בת מהדוח הגולמי, לפי מוסכמת עבודה. סה"כ שורת "Total" בדוח הגולמי המלא: ₪58,251.29 - תואם בדיוק לסכום 2 שורות הקטגוריה שנשלפו (₪27,768.00+₪30,483.29=₪58,251.29, אומת ידנית).</t>
   </si>
   <si>
     <t xml:space="preserve">Customer</t>
@@ -315,7 +315,7 @@
     <t xml:space="preserve">Sales</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: צילום מסך/נתונים שסופקו על ידי המשתמש (ראובן), לוח בקרה Sellerboard/Amazon Seller "Month to date, 1-30 September 2026" (חודש ספטמבר שלם), נמסר במקור 01/10/2026 עבור דוח 01/10/2026, מאומת בטקסט (לא תמלול תמונה). עדכון 04/10/2026: לא סופק צילום מסך חדש לדוח זה — לפי בקשה מפורשת של המשתמש, נעשה שימוש חוזר (recycle) באותם נתוני ספטמבר המלא (Sales $71,888.24, Refund cost -$5,648.73) ששימשו בדוח 01/10/2026, שגם הוא היה סגירת ספטמבר. אין נתון Amazon חדש/עצמאי לדוח 04/10/2026 עצמו. נתונים נוספים שסופקו במקור (לא בשימוש בנוסחה): Sales -1.6% מול תקופה קודמת, Orders/Units 2,299/2,349, Refunds 203, Est. payout $24,338.36, Gross profit $10,785.13, Net profit $10,785.13 -10.9% (זהה ל-Gross profit, כפי שמופיע במקור).</t>
+    <t xml:space="preserve">Source: צילום מסך/נתונים שסופקו על ידי המשתמש (ראובן), לוח בקרה Sellerboard/Amazon Seller "Month to date, 1-3 October 2026" (3 ימים לתוך החודש החדש), נמסר 04/10/2026 עבור דוח 04/10/2026, מאומת בטקסט (לא תמלול תמונה). נתונים נוספים שסופקו במקור (לא בשימוש בנוסחה): Sales +37.0% מול תקופה קודמת, Orders/Units 268/279, Refunds 27, Est. payout $2,839.48, Gross profit $1,370.93, Net profit $1,370.93 +32.6% (זהה ל-Gross profit, כפי שמופיע במקור).</t>
   </si>
   <si>
     <t xml:space="preserve">תיאור</t>
@@ -324,13 +324,13 @@
     <t xml:space="preserve">סכום ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">משמש בנוסחת 'סהכ'!C20: =(Sales+Refund cost)×3. נתון מחזור (recycled) מדוח 01/10/2026 — אין צילום מסך חדש לדוח זה.</t>
+    <t xml:space="preserve">משמש בנוסחת 'סהכ'!C20: =(Sales+Refund cost)×3.</t>
   </si>
   <si>
     <t xml:space="preserve">Refund cost</t>
   </si>
   <si>
-    <t xml:space="preserve">מכפיל ×3 לפי הנחיית המשתמש (לא מתועד במקור התמונה). נתון מחזור (recycled) מדוח 01/10/2026 — אין צילום מסך חדש לדוח זה.</t>
+    <t xml:space="preserve">מכפיל ×3 לפי הנחיית המשתמש (לא מתועד במקור התמונה).</t>
   </si>
 </sst>
 </file>
@@ -974,7 +974,7 @@
         <v>46299</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>9.2026</v>
+        <v>10.2026</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -986,7 +986,7 @@
       </c>
       <c r="C3" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A3,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A3,ריכוז!$C$3:$C$30)</f>
-        <v>193941.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -998,7 +998,7 @@
       </c>
       <c r="C4" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A4,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A4,ריכוז!$C$3:$C$30)</f>
-        <v>507718.575</v>
+        <v>6919.185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A5,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A5,ריכוז!$C$3:$C$30)</f>
-        <v>73475.311</v>
+        <v>1693.51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A6,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A6,ריכוז!$C$3:$C$30)</f>
-        <v>182488.743</v>
+        <v>1518.153</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A7,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A7,ריכוז!$C$3:$C$30)</f>
-        <v>296928.1</v>
+        <v>27768</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A8,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A8,ריכוז!$C$3:$C$30)</f>
-        <v>55452.215</v>
+        <v>803.621</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A9,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A9,ריכוז!$C$3:$C$30)</f>
-        <v>60353.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A10,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A10,ריכוז!$C$3:$C$30)</f>
-        <v>8627.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A11,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A11,ריכוז!$C$3:$C$30)</f>
-        <v>5091.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A14,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A14,ריכוז!$C$3:$C$30)</f>
-        <v>6726.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A15,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A15,ריכוז!$C$3:$C$30)</f>
-        <v>9421.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="C16" s="15" t="n">
         <f aca="false">SUM(C3:C15)</f>
-        <v>1400225.374</v>
+        <v>38702.469</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A17,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A17,ריכוז!$C$3:$C$30)</f>
-        <v>347579.04</v>
+        <v>30483.29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C18" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A18,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A18,ריכוז!$C$3:$C$30)</f>
-        <v>547.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="C19" s="15" t="n">
         <f aca="false">C18+C17+C16</f>
-        <v>1748351.434</v>
+        <v>69185.759</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="C20" s="9" t="n">
         <f aca="false">(Amazon_מקור!B3+Amazon_מקור!B4)*3</f>
-        <v>198718.53</v>
+        <v>22723.8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A23,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A23,ריכוז!$C$3:$C$30)</f>
-        <v>51223.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A24,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A24,ריכוז!$C$3:$C$30)</f>
-        <v>15160.58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A29,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A29,ריכוז!$C$3:$C$30)</f>
-        <v>25430.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C31" s="9" t="n">
         <f aca="false">SUMIF(Pplay1!$F$3:$F$15,A31,Pplay1!$H$3:$H$15)+SUMIF(ריכוז!$B$3:$B$30,A31,ריכוז!$C$3:$C$30)</f>
-        <v>21590.63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C40" s="18" t="n">
         <f aca="false">SUM(C20:C39)</f>
-        <v>312123.16</v>
+        <v>22723.8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="C41" s="20" t="n">
         <f aca="false">C40+C19</f>
-        <v>2060474.594</v>
+        <v>91909.559</v>
       </c>
     </row>
   </sheetData>
@@ -1507,11 +1507,11 @@
       </c>
       <c r="G3" s="27" t="n">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A3,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>186065.8</v>
+        <v>1953</v>
       </c>
       <c r="H3" s="27" t="n">
         <f aca="false">IF(G3="","",G3*0.91)</f>
-        <v>169319.878</v>
+        <v>1777.23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1528,13 +1528,13 @@
         <f aca="false">IF(B4&lt;&gt;"",B4,IF(C4&lt;&gt;"",C4,IF(D4&lt;&gt;"",D4,IF(E4&lt;&gt;"",E4,""))))</f>
         <v>4</v>
       </c>
-      <c r="G4" s="27" t="n">
+      <c r="G4" s="27" t="str">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A4,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>577.7</v>
-      </c>
-      <c r="H4" s="27" t="n">
+        <v/>
+      </c>
+      <c r="H4" s="27" t="str">
         <f aca="false">IF(G4="","",G4*0.91)</f>
-        <v>525.707</v>
+        <v/>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1551,11 +1551,11 @@
       </c>
       <c r="G5" s="27" t="n">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A5,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>639577.2</v>
+        <v>9179.8</v>
       </c>
       <c r="H5" s="27" t="n">
         <f aca="false">IF(G5="","",G5*0.91)</f>
-        <v>582015.252</v>
+        <v>8353.618</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1572,13 +1572,13 @@
         <f aca="false">IF(B6&lt;&gt;"",B6,IF(C6&lt;&gt;"",C6,IF(D6&lt;&gt;"",D6,IF(E6&lt;&gt;"",E6,""))))</f>
         <v>7</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="27" t="str">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A6,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>6632</v>
-      </c>
-      <c r="H6" s="27" t="n">
+        <v/>
+      </c>
+      <c r="H6" s="27" t="str">
         <f aca="false">IF(G6="","",G6*0.91)</f>
-        <v>6035.12</v>
+        <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1595,13 +1595,13 @@
         <f aca="false">IF(B7&lt;&gt;"",B7,IF(C7&lt;&gt;"",C7,IF(D7&lt;&gt;"",D7,IF(E7&lt;&gt;"",E7,""))))</f>
         <v>4</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="27" t="str">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A7,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>902.8</v>
-      </c>
-      <c r="H7" s="27" t="n">
+        <v/>
+      </c>
+      <c r="H7" s="27" t="str">
         <f aca="false">IF(G7="","",G7*0.91)</f>
-        <v>821.548</v>
+        <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1618,13 +1618,13 @@
         <f aca="false">IF(B8&lt;&gt;"",B8,IF(C8&lt;&gt;"",C8,IF(D8&lt;&gt;"",D8,IF(E8&lt;&gt;"",E8,""))))</f>
         <v>4</v>
       </c>
-      <c r="G8" s="27" t="str">
+      <c r="G8" s="27" t="n">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A8,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H8" s="27" t="str">
+        <v>-284.7</v>
+      </c>
+      <c r="H8" s="27" t="n">
         <f aca="false">IF(G8="","",G8*0.91)</f>
-        <v/>
+        <v>-259.077</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1641,13 +1641,13 @@
         <f aca="false">IF(B9&lt;&gt;"",B9,IF(C9&lt;&gt;"",C9,IF(D9&lt;&gt;"",D9,IF(E9&lt;&gt;"",E9,""))))</f>
         <v>7</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="27" t="str">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A9,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>362.9</v>
-      </c>
-      <c r="H9" s="27" t="n">
+        <v/>
+      </c>
+      <c r="H9" s="27" t="str">
         <f aca="false">IF(G9="","",G9*0.91)</f>
-        <v>330.239</v>
+        <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1666,11 +1666,11 @@
       </c>
       <c r="G10" s="27" t="n">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A10,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>557932.5</v>
+        <v>7603.5</v>
       </c>
       <c r="H10" s="27" t="n">
         <f aca="false">IF(G10="","",G10*0.91)</f>
-        <v>507718.575</v>
+        <v>6919.185</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1689,11 +1689,11 @@
       </c>
       <c r="G11" s="27" t="n">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A11,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>74555.9</v>
+        <v>1861</v>
       </c>
       <c r="H11" s="27" t="n">
         <f aca="false">IF(G11="","",G11*0.91)</f>
-        <v>67845.869</v>
+        <v>1693.51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1735,11 +1735,11 @@
       </c>
       <c r="G13" s="27" t="n">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A13,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>60936.5</v>
+        <v>883.1</v>
       </c>
       <c r="H13" s="27" t="n">
         <f aca="false">IF(G13="","",G13*0.91)</f>
-        <v>55452.215</v>
+        <v>803.621</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1779,13 +1779,13 @@
         <f aca="false">IF(B15&lt;&gt;"",B15,IF(C15&lt;&gt;"",C15,IF(D15&lt;&gt;"",D15,IF(E15&lt;&gt;"",E15,""))))</f>
         <v>7</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="27" t="str">
         <f aca="false">IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A15,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v>-808.7</v>
-      </c>
-      <c r="H15" s="27" t="n">
+        <v/>
+      </c>
+      <c r="H15" s="27" t="str">
         <f aca="false">IF(G15="","",G15*0.91)</f>
-        <v>-735.917</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1829,9 +1829,9 @@
       <c r="B3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C3" s="27" t="n">
+      <c r="C3" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A3,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>60353.17</v>
+        <v/>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1841,9 +1841,9 @@
       <c r="B4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="27" t="n">
+      <c r="C4" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A4,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>193941.5</v>
+        <v/>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1853,9 +1853,9 @@
       <c r="B5" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A5,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>9421.74</v>
+        <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1865,9 +1865,9 @@
       <c r="B6" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A6,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>5091.7</v>
+        <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1877,9 +1877,9 @@
       <c r="B7" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A7,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>8627.76</v>
+        <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1889,9 +1889,9 @@
       <c r="B8" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A8,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>11821.61</v>
+        <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1901,9 +1901,9 @@
       <c r="B9" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A9,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>6726.56</v>
+        <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="C11" s="27" t="n">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A11,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>296928.1</v>
+        <v>27768</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="C12" s="27" t="n">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A12,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>347579.04</v>
+        <v>30483.29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1949,9 +1949,9 @@
       <c r="B13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A13,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>547.02</v>
+        <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1961,9 +1961,9 @@
       <c r="B14" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A14,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>15160.58</v>
+        <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1985,9 +1985,9 @@
       <c r="B16" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="27" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A16,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>25430.19</v>
+        <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2033,9 +2033,9 @@
       <c r="B20" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="C20" s="29" t="n">
+      <c r="C20" s="29" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A20,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>51223.23</v>
+        <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2093,9 +2093,9 @@
       <c r="B25" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="C25" s="29" t="n">
+      <c r="C25" s="29" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A25,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v>21590.63</v>
+        <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2202,128 +2202,96 @@
         <v>48</v>
       </c>
       <c r="B2" s="27" t="n">
-        <v>186065.8</v>
+        <v>1953</v>
       </c>
       <c r="C2" s="27" t="n">
         <f aca="false">B2*0.91</f>
-        <v>169319.878</v>
+        <v>1777.23</v>
       </c>
       <c r="D2" s="30"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B3" s="27" t="n">
-        <v>577.7</v>
+        <v>9179.8</v>
       </c>
       <c r="C3" s="27" t="n">
         <f aca="false">B3*0.91</f>
-        <v>525.707</v>
+        <v>8353.618</v>
       </c>
       <c r="D3" s="30"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B4" s="27" t="n">
-        <v>639577.2</v>
+        <v>-284.7</v>
       </c>
       <c r="C4" s="27" t="n">
         <f aca="false">B4*0.91</f>
-        <v>582015.252</v>
+        <v>-259.077</v>
       </c>
       <c r="D4" s="30"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6632</v>
+        <v>7603.5</v>
       </c>
       <c r="C5" s="27" t="n">
         <f aca="false">B5*0.91</f>
-        <v>6035.12</v>
+        <v>6919.185</v>
       </c>
       <c r="D5" s="30"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" s="27" t="n">
-        <v>362.9</v>
+        <v>1861</v>
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">B6*0.91</f>
-        <v>330.239</v>
+        <v>1693.51</v>
       </c>
       <c r="D6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B7" s="27" t="n">
-        <v>-808.7</v>
+        <v>883.1</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">B7*0.91</f>
-        <v>-735.917</v>
+        <v>803.621</v>
       </c>
       <c r="D7" s="30"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="27" t="n">
-        <v>557932.5</v>
-      </c>
-      <c r="C8" s="27" t="n">
-        <f aca="false">B8*0.91</f>
-        <v>507718.575</v>
-      </c>
+      <c r="A8" s="26"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
       <c r="D8" s="30"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="27" t="n">
-        <v>74555.9</v>
-      </c>
-      <c r="C9" s="27" t="n">
-        <f aca="false">B9*0.91</f>
-        <v>67845.869</v>
-      </c>
+      <c r="A9" s="26"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="27" t="n">
-        <v>60936.5</v>
-      </c>
-      <c r="C10" s="27" t="n">
-        <f aca="false">B10*0.91</f>
-        <v>55452.215</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>902.8</v>
-      </c>
-      <c r="C11" s="1" t="n">
-        <f aca="false">B11*0.91</f>
-        <v>821.548</v>
-      </c>
-    </row>
+      <c r="A10" s="26"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2362,121 +2330,73 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D3" s="29" t="n">
-        <v>60353.17</v>
+        <v>27768</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D4" s="29" t="n">
-        <v>9421.74</v>
+        <v>30483.29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="29" t="n">
-        <v>5091.7</v>
-      </c>
+      <c r="A5" s="26"/>
+      <c r="D5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" s="29" t="n">
-        <v>193941.5</v>
-      </c>
+      <c r="A6" s="26"/>
+      <c r="D6" s="29"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="29" t="n">
-        <v>8627.76</v>
-      </c>
+      <c r="A7" s="26"/>
+      <c r="D7" s="29"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="D8" s="29" t="n">
-        <v>11821.61</v>
-      </c>
+      <c r="A8" s="26"/>
+      <c r="D8" s="29"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" s="29" t="n">
-        <v>296928.1</v>
-      </c>
+      <c r="A9" s="26"/>
+      <c r="D9" s="29"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="D10" s="29" t="n">
-        <v>347579.04</v>
-      </c>
+      <c r="A10" s="26"/>
+      <c r="D10" s="29"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="29" t="n">
-        <v>547.02</v>
-      </c>
+      <c r="A11" s="26"/>
+      <c r="D11" s="29"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="26" t="s">
-        <v>73</v>
-      </c>
+      <c r="A12" s="26"/>
       <c r="B12" s="31"/>
       <c r="C12" s="31"/>
-      <c r="D12" s="29" t="n">
-        <v>15160.58</v>
-      </c>
+      <c r="D12" s="29"/>
       <c r="E12" s="32"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="33" t="s">
-        <v>75</v>
-      </c>
+      <c r="A13" s="33"/>
       <c r="B13" s="31"/>
       <c r="C13" s="31"/>
-      <c r="D13" s="34" t="n">
-        <v>25430.19</v>
-      </c>
+      <c r="D13" s="34"/>
       <c r="E13" s="32"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" s="27" t="n">
-        <v>51223.23</v>
-      </c>
+      <c r="A14" s="26"/>
+      <c r="D14" s="27"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" s="27" t="n">
-        <v>6726.56</v>
-      </c>
+      <c r="A15" s="26"/>
+      <c r="D15" s="27"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="26" t="s">
-        <v>84</v>
-      </c>
-      <c r="D16" s="27" t="n">
-        <v>21590.63</v>
-      </c>
+      <c r="A16" s="26"/>
+      <c r="D16" s="27"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2525,7 +2445,7 @@
         <v>95</v>
       </c>
       <c r="B3" s="27" t="n">
-        <v>71888.24</v>
+        <v>8443.05</v>
       </c>
       <c r="C3" s="30" t="s">
         <v>99</v>
@@ -2536,7 +2456,7 @@
         <v>100</v>
       </c>
       <c r="B4" s="27" t="n">
-        <v>-5648.73</v>
+        <v>-868.45</v>
       </c>
       <c r="C4" s="30" t="s">
         <v>101</v>

</xml_diff>